<commit_message>
chore: checkpoint development work in progress
Save current in-progress changes to continue tomorrow on development.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/ShelfMind-RPA/downloads/gvVendedores.xlsx
+++ b/ShelfMind-RPA/downloads/gvVendedores.xlsx
@@ -46,12 +46,28 @@
   <si>
     <t>Bat. ultima</t>
   </si>
+  <si>
+    <t>d85448b306cc3029</t>
+  </si>
+  <si>
+    <t>miguel diduch</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> MIGUEL DIDUCH</t>
+  </si>
+  <si>
+    <t>6.2.11</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="HH:mm"/>
+    <numFmt numFmtId="165" formatCode="0.##"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -64,8 +80,13 @@
       <color rgb="FFFFFFFF"/>
       <name val="Times New Roman"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -75,6 +96,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF808080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -105,16 +131,61 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" shrinkToFit="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="609600" cy="400050"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -384,11 +455,11 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <cols>
-    <col min="1" max="1" width="4.14" customWidth="1"/>
-    <col min="2" max="2" width="4.71" customWidth="1"/>
-    <col min="3" max="3" width="9.71" customWidth="1"/>
+    <col min="1" max="1" width="15.43" customWidth="1"/>
+    <col min="2" max="2" width="11.43" customWidth="1"/>
+    <col min="3" max="3" width="16.14" customWidth="1"/>
     <col min="4" max="4" width="7.43" customWidth="1"/>
-    <col min="5" max="5" width="5.86" customWidth="1"/>
+    <col min="5" max="5" width="9.43" customWidth="1"/>
     <col min="6" max="6" width="10.29" customWidth="1"/>
     <col min="7" max="7" width="9" customWidth="1"/>
     <col min="8" max="8" width="7.86" customWidth="1"/>
@@ -436,11 +507,46 @@
         <v>11</v>
       </c>
     </row>
+    <row r="2" ht="33" customHeight="1">
+      <c t="s" r="A2" s="2">
+        <v>12</v>
+      </c>
+      <c t="s" r="B2" s="2">
+        <v>13</v>
+      </c>
+      <c t="s" r="C2" s="2">
+        <v>14</v>
+      </c>
+      <c r="D2" s="2"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="4">
+        <v>46110.822175925925</v>
+      </c>
+      <c r="G2" s="4">
+        <v>46110.822430555556</v>
+      </c>
+      <c r="H2" s="5">
+        <v>3</v>
+      </c>
+      <c r="I2" s="5">
+        <v>0</v>
+      </c>
+      <c t="s" r="J2" s="2">
+        <v>15</v>
+      </c>
+      <c r="K2" s="6">
+        <v>0</v>
+      </c>
+      <c r="L2" s="6">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:L1" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:L2" numberStoredAsText="1"/>
   </ignoredErrors>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: watcher conversion_estado logic and portal feedback permissions
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ShelfMind-RPA/downloads/gvVendedores.xlsx
+++ b/ShelfMind-RPA/downloads/gvVendedores.xlsx
@@ -46,28 +46,12 @@
   <si>
     <t>Bat. ultima</t>
   </si>
-  <si>
-    <t>d85448b306cc3029</t>
-  </si>
-  <si>
-    <t>miguel diduch</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> MIGUEL DIDUCH</t>
-  </si>
-  <si>
-    <t>6.2.11</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="HH:mm"/>
-    <numFmt numFmtId="165" formatCode="0.##"/>
-  </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -80,13 +64,8 @@
       <color rgb="FFFFFFFF"/>
       <name val="Times New Roman"/>
     </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -96,11 +75,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF808080"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -131,61 +105,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1" shrinkToFit="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="609600" cy="400050"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect"/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -455,11 +384,11 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <cols>
-    <col min="1" max="1" width="15.43" customWidth="1"/>
-    <col min="2" max="2" width="11.43" customWidth="1"/>
-    <col min="3" max="3" width="16.14" customWidth="1"/>
+    <col min="1" max="1" width="4.14" customWidth="1"/>
+    <col min="2" max="2" width="4.71" customWidth="1"/>
+    <col min="3" max="3" width="9.71" customWidth="1"/>
     <col min="4" max="4" width="7.43" customWidth="1"/>
-    <col min="5" max="5" width="9.43" customWidth="1"/>
+    <col min="5" max="5" width="5.86" customWidth="1"/>
     <col min="6" max="6" width="10.29" customWidth="1"/>
     <col min="7" max="7" width="9" customWidth="1"/>
     <col min="8" max="8" width="7.86" customWidth="1"/>
@@ -507,46 +436,11 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" ht="33" customHeight="1">
-      <c t="s" r="A2" s="2">
-        <v>12</v>
-      </c>
-      <c t="s" r="B2" s="2">
-        <v>13</v>
-      </c>
-      <c t="s" r="C2" s="2">
-        <v>14</v>
-      </c>
-      <c r="D2" s="2"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="4">
-        <v>46110.822175925925</v>
-      </c>
-      <c r="G2" s="4">
-        <v>46110.822430555556</v>
-      </c>
-      <c r="H2" s="5">
-        <v>3</v>
-      </c>
-      <c r="I2" s="5">
-        <v>0</v>
-      </c>
-      <c t="s" r="J2" s="2">
-        <v>15</v>
-      </c>
-      <c r="K2" s="6">
-        <v>0</v>
-      </c>
-      <c r="L2" s="6">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:L2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:L1" numberStoredAsText="1"/>
   </ignoredErrors>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>